<commit_message>
feat: add defect tracking analytic sheet
</commit_message>
<xml_diff>
--- a/CS341_A1_DefectTracker_Group5.xlsx
+++ b/CS341_A1_DefectTracker_Group5.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHIVAN\Desktop\CS341\Assignment 1\A1\A1 Final\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aryan\OneDrive\Desktop\S2 2026\ASG\CS341\A1\CS341_A1_Java_Starter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9483A811-F5FB-4181-B5AA-B545D48D6DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{360A2AC3-A1EA-4750-94BD-C4079AD7D015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,9 +20,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -75,6 +72,85 @@
     <t>Hours above the maximum valid range are accepted for Visitor car.</t>
   </si>
   <si>
+    <t>DF-03</t>
+  </si>
+  <si>
+    <t>TC20</t>
+  </si>
+  <si>
+    <t>Resident car charger at exactly 12 hours is incorrect</t>
+  </si>
+  <si>
+    <t>DF-04</t>
+  </si>
+  <si>
+    <t>TC29</t>
+  </si>
+  <si>
+    <t>Hours above the maximum valid range are accepted for Trucks.</t>
+  </si>
+  <si>
+    <t>DF-05</t>
+  </si>
+  <si>
+    <t>TC34</t>
+  </si>
+  <si>
+    <t>Truck is accepting a permit value below the valid range</t>
+  </si>
+  <si>
+    <t>DF-06</t>
+  </si>
+  <si>
+    <t>TC35</t>
+  </si>
+  <si>
+    <t>Truck is accepting a permit value above the valid range</t>
+  </si>
+  <si>
+    <t>Updated Status</t>
+  </si>
+  <si>
+    <t>Updated Resolution</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>The Visitor charging boundary was corrected so that the $4.00 per hour tier ends
+ at 12 hours and the $8.00 per hour tier begins at 13 hours, 
+after being retested, it returned 104.00 as expected.</t>
+  </si>
+  <si>
+    <t>For hoursOverstayed values greater than 48 validation is added.
+ TC16 was retested with 49 hours and it returned -1 as expected</t>
+  </si>
+  <si>
+    <t>The Resident charging boundary was corrected so that 12 hours remain in the $1.00 per hour tier.
+ TC20 was retested and it returned 12.00 as expected.</t>
+  </si>
+  <si>
+    <t>For hoursOverstayed values greater than 48 validation was added, before calculating the Truck charge. 
+TC29 was retested and it returned -1 as expected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moved the permit validation before the calculation of Truck charge. 
+TC34 was retested with permitType = 0 and it returned -1. </t>
+  </si>
+  <si>
+    <t>Moved the permit validation before the calculation of Truck charge. 
+TC35 was retested with permitType = 3 and it returned -1 as expected.</t>
+  </si>
+  <si>
+    <t>Major/High</t>
+  </si>
+  <si>
+    <t>Needs correction and retest will be done in Task 6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Correction is needed and retest will be done in Task 6.</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -135,7 +211,7 @@
         <family val="1"/>
       </rPr>
       <t xml:space="preserve"> 
-1. Run computeOverstayCharger 13, 1, 1)
+1. Run computeOverstayCharge 49, 1, 1)
 2. Record the returned charge
 3. Compare the results with the valid hour range given in the specification.
 </t>
@@ -184,13 +260,113 @@
     </r>
   </si>
   <si>
-    <t>DF-03</t>
-  </si>
-  <si>
-    <t>TC20</t>
-  </si>
-  <si>
-    <t>Resident car charger at exactly 12 hours is incorrect</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Precondition:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+The original given CalOverstayCharge implementation was used.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Inputs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">:
+hoursOverStayed = 13, vehicleType = 1 (Car), permitType = 1 (Visitors)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Steps to reproduce:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 
+1. Run computeOverstayCharge 13, 1, 1)
+2. Record the returned charge
+3. Compare the results with the car charging rule for Visitors.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Expected Result:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 
+$104.00. Visitor car overstaying for 13 is charged 8.00 per hours, thus 13 * 8.00 = 104.00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Actual Result: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">52.00
+The charge returned is lower than expected at the 13-hour boundary.
+</t>
+    </r>
   </si>
   <si>
     <r>
@@ -253,7 +429,7 @@
         <family val="1"/>
       </rPr>
       <t xml:space="preserve">
-1. Run computeOverstayCharger 12, 1, 2)
+1. Run computeOverstayCharge 12, 1, 2)
 2. Record the returned charge
 3. Compare the results with the Resident care charging rules.
 </t>
@@ -302,15 +478,6 @@
     </r>
   </si>
   <si>
-    <t>DF-04</t>
-  </si>
-  <si>
-    <t>TC29</t>
-  </si>
-  <si>
-    <t>Hours above the maximum valid range are accepted for Trucks.</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -371,7 +538,7 @@
         <family val="1"/>
       </rPr>
       <t xml:space="preserve">
-1. Run computeOverstayCharger (49, 2, 1)
+1. Run computeOverstayCharge (49, 2, 1)
 2. Record the returned charge
 3. Compare the results with the valid hour ranges.
 </t>
@@ -420,15 +587,6 @@
     </r>
   </si>
   <si>
-    <t>DF-05</t>
-  </si>
-  <si>
-    <t>TC34</t>
-  </si>
-  <si>
-    <t>Truck is accepting a permit value below the valid range</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -489,7 +647,7 @@
         <family val="1"/>
       </rPr>
       <t xml:space="preserve"> 
-1. Run computeOverstayCharger (5, 2, 0)
+1. Run computeOverstayCharge (5, 2, 0)
 2. Record the returned charge
 3. Compare the results with the permitted input values.
 </t>
@@ -536,15 +694,6 @@
       <t>75.00
 Program calculates the charge even though the permit input is invalid.</t>
     </r>
-  </si>
-  <si>
-    <t>DF-06</t>
-  </si>
-  <si>
-    <t>TC35</t>
-  </si>
-  <si>
-    <t>Truck is accepting a permit value above the valid range</t>
   </si>
   <si>
     <t>Precondition:
@@ -552,7 +701,7 @@
 Inputs:
 hoursOverStayed = 5, vehicleType = 2 (Truck), permitType = 3
 Steps to reproduce: 
-1. Run computeOverstayCharger (5, 2, 0)
+1. Run computeOverstayCharge (5, 2, 3)
 2. Record the returned charge
 3. Compare the results with the permitted input values.
 Expected Result: 
@@ -560,158 +709,6 @@
 Actual Result:
 75.00
 Program calculates the Truck charge even though the permit input is invalid.</t>
-  </si>
-  <si>
-    <t>Updated Status</t>
-  </si>
-  <si>
-    <t>Updated Resolution</t>
-  </si>
-  <si>
-    <t>Closed</t>
-  </si>
-  <si>
-    <t>The Visitor charging boundary was corrected so that the $4.00 per hour tier ends
- at 12 hours and the $8.00 per hour tier begins at 13 hours, 
-after being retested, it returned 104.00 as expected.</t>
-  </si>
-  <si>
-    <t>For hoursOverstayed values greater than 48 validation is added.
- TC16 was retested with 49 hours and it returned -1 as expected</t>
-  </si>
-  <si>
-    <t>The Resident charging boundary was corrected so that 12 hours remain in the $1.00 per hour tier.
- TC20 was retested and it returned 12.00 as expected.</t>
-  </si>
-  <si>
-    <t>For hoursOverstayed values greater than 48 validation was added, before calculating the Truck charge. 
-TC29 was retested and it returned -1 as expected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moved the permit validation before the calculation of Truck charge. 
-TC34 was retested with permitType = 0 and it returned -1. </t>
-  </si>
-  <si>
-    <t>Moved the permit validation before the calculation of Truck charge. 
-TC35 was retested with permitType = 3 and it returned -1 as expected.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Precondition:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">
-The original given CalOverstayCharge implementation was used.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Inputs</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">:
-hoursOverStayed = 13, vehicleType = 1 (Car), permitType = 1 (Visitors)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Steps to reproduce:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 
-1. Run computeOverstayCharger 13, 1, 1)
-2. Record the returned charge
-3. Compare the results with the car charging rule for Visitors.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Expected Result:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 
-$104.00. Visitor car overstaying for 13 is charged 8.00 per hours, thus 13 * 8.00 = 104.00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">Actual Result: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">52.00
-The charge returned is lower than expected at the 13-hour boundary.
-</t>
-    </r>
-  </si>
-  <si>
-    <t>Major/High</t>
-  </si>
-  <si>
-    <t>Needs correction and retest will be done in Task 6.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Correction is needed and retest will be done in Task 6.</t>
   </si>
 </sst>
 </file>
@@ -1091,13 +1088,13 @@
         <v>6</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="2" spans="2:11" s="1" customFormat="1" ht="196" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:11" s="1" customFormat="1" ht="210" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1108,10 +1105,10 @@
         <v>9</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>10</v>
@@ -1120,13 +1117,13 @@
         <v>11</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
-    <row r="3" spans="2:11" s="1" customFormat="1" ht="210" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:11" s="1" customFormat="1" ht="224" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1137,39 +1134,39 @@
         <v>14</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="K3" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" s="1" customFormat="1" ht="210" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="2:11" s="1" customFormat="1" ht="196" x14ac:dyDescent="0.3">
-      <c r="B4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>10</v>
@@ -1178,27 +1175,27 @@
         <v>11</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="2:11" s="1" customFormat="1" ht="210" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="E5" s="3" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>10</v>
@@ -1207,56 +1204,56 @@
         <v>11</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="2:11" s="1" customFormat="1" ht="196" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="J6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="2:11" s="1" customFormat="1" ht="210" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>10</v>
@@ -1265,10 +1262,10 @@
         <v>11</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="2:11" s="1" customFormat="1" ht="14" x14ac:dyDescent="0.3"/>

</xml_diff>